<commit_message>
bug free code was added
</commit_message>
<xml_diff>
--- a/basket/sub_frames.xlsx
+++ b/basket/sub_frames.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>SubFrame</t>
   </si>
@@ -17,22 +17,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>[e2, 0, 0, 1d, 43, f, 2, 0, 13, 60, ad, 40]</t>
+    <t>[e2, 0, 34, 12, 1, 33, ff, 0, 0, 26, 99, 7f]</t>
   </si>
   <si>
     <t>1</t>
-  </si>
-  <si>
-    <t>[e2, 0, 34, 12, 1, 33, ff, 0, 0, 26, 99, 7e]</t>
-  </si>
-  <si>
-    <t>[30, 8, 33, b2, dd, d9, 1, 40, 0, 0, 0, 0]</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>[e2, 0, 34, 12, 1, 33, ff, 0, 0, 26, 99, 7f]</t>
   </si>
 </sst>
 </file>
@@ -420,30 +408,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>